<commit_message>
test(import): make multi-currency sample produce consistent records
The sample only had a Total column, so imported revenues/expenses got a 0 Unit Price and a 0 line item while Total was set, which made the edit modal show 0 and warn about a mismatch. Add a Unit Price column (qty 1, so Unit Price == Total) so the line item matches the total and the record is internally consistent. Strengthen the regression test to assert Amount == Total.

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/TestData/MainImporter/multi_currency_sample.xlsx
+++ b/TestData/MainImporter/multi_currency_sample.xlsx
@@ -426,7 +426,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,6 +452,11 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
@@ -480,6 +485,9 @@
       <c r="E2" s="1" t="n">
         <v>1200</v>
       </c>
+      <c r="F2" s="1" t="n">
+        <v>1200</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -505,6 +513,9 @@
       <c r="E3" s="2" t="n">
         <v>800</v>
       </c>
+      <c r="F3" s="2" t="n">
+        <v>800</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -530,6 +541,9 @@
       <c r="E4" s="3" t="n">
         <v>1500</v>
       </c>
+      <c r="F4" s="3" t="n">
+        <v>1500</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -555,6 +569,9 @@
       <c r="E5" s="4" t="n">
         <v>95000</v>
       </c>
+      <c r="F5" s="4" t="n">
+        <v>95000</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -580,6 +597,9 @@
       <c r="E6" s="5" t="n">
         <v>950</v>
       </c>
+      <c r="F6" s="5" t="n">
+        <v>950</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -603,6 +623,9 @@
         </is>
       </c>
       <c r="E7" s="6" t="n">
+        <v>500</v>
+      </c>
+      <c r="F7" s="6" t="n">
         <v>500</v>
       </c>
     </row>
@@ -617,7 +640,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:F5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -643,6 +666,11 @@
       </c>
       <c r="E1" t="inlineStr">
         <is>
+          <t>Unit Price</t>
+        </is>
+      </c>
+      <c r="F1" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
@@ -671,6 +699,9 @@
       <c r="E2" s="1" t="n">
         <v>140</v>
       </c>
+      <c r="F2" s="1" t="n">
+        <v>140</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -696,6 +727,9 @@
       <c r="E3" s="3" t="n">
         <v>320</v>
       </c>
+      <c r="F3" s="3" t="n">
+        <v>320</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -721,6 +755,9 @@
       <c r="E4" s="5" t="n">
         <v>88</v>
       </c>
+      <c r="F4" s="5" t="n">
+        <v>88</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -744,6 +781,9 @@
         </is>
       </c>
       <c r="E5" s="6" t="n">
+        <v>1500</v>
+      </c>
+      <c r="F5" s="6" t="n">
         <v>1500</v>
       </c>
     </row>

</xml_diff>